<commit_message>
controller design first commit
</commit_message>
<xml_diff>
--- a/files/Plan.xlsx
+++ b/files/Plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulisboa-my.sharepoint.com/personal/ist1100262_tecnico_ulisboa_pt/Documents/MEMec/Thesis/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{733EBFC7-8944-45D8-B0FC-2B9A37E95772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75C01B61-87B5-4D75-803D-1822565DCCD9}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{733EBFC7-8944-45D8-B0FC-2B9A37E95772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02B98C8A-250B-442C-B437-12B9304D5DD0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{563C961A-BFB9-4F7A-BA15-8C34454DAF79}"/>
+    <workbookView xWindow="2352" yWindow="924" windowWidth="17268" windowHeight="9372" xr2:uid="{563C961A-BFB9-4F7A-BA15-8C34454DAF79}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -404,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -448,6 +448,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -464,15 +467,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -819,46 +813,46 @@
   <sheetData>
     <row r="1" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B2" s="20"/>
-      <c r="C2" s="22" t="s">
+      <c r="B2" s="21"/>
+      <c r="C2" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="17" t="s">
+      <c r="D2" s="19"/>
+      <c r="E2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="17" t="s">
+      <c r="F2" s="19"/>
+      <c r="G2" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="18"/>
-      <c r="I2" s="17" t="s">
+      <c r="H2" s="19"/>
+      <c r="I2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="18"/>
-      <c r="K2" s="17" t="s">
+      <c r="J2" s="19"/>
+      <c r="K2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="18"/>
-      <c r="M2" s="17" t="s">
+      <c r="L2" s="19"/>
+      <c r="M2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="18"/>
-      <c r="O2" s="17" t="s">
+      <c r="N2" s="19"/>
+      <c r="O2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="17" t="s">
+      <c r="P2" s="19"/>
+      <c r="Q2" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="18"/>
-      <c r="S2" s="17" t="s">
+      <c r="R2" s="19"/>
+      <c r="S2" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="T2" s="19"/>
+      <c r="T2" s="20"/>
     </row>
     <row r="3" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="21"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="9">
         <v>1</v>
       </c>
@@ -1106,7 +1100,7 @@
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="14"/>
-      <c r="G12" s="23"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -1128,7 +1122,7 @@
       <c r="C13" s="1"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="23"/>
+      <c r="F13" s="2"/>
       <c r="G13" s="14"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -1151,7 +1145,7 @@
       <c r="C14" s="1"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="23"/>
+      <c r="F14" s="2"/>
       <c r="G14" s="14"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -1177,7 +1171,7 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="14"/>
-      <c r="I15" s="2"/>
+      <c r="I15" s="14"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1201,7 +1195,7 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+      <c r="J16" s="14"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
@@ -1225,8 +1219,8 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -1240,9 +1234,9 @@
       <c r="B18" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
       <c r="H18" s="15"/>

</xml_diff>